<commit_message>
test: align syllabus sample files and demo data with the new Sheet 1 form
</commit_message>
<xml_diff>
--- a/docs/mau-test-kho-syllabus/cap-nhat-starters-chang-1.xlsx
+++ b/docs/mau-test-kho-syllabus/cap-nhat-starters-chang-1.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="64">
   <si>
     <t>SYLLABUS MẪU – FORM CHUẨN CỦA HỌC THUẬT</t>
   </si>
   <si>
-    <t>Mỗi file = 1 chặng của 1 giáo trình. Ô nền vàng là ô cần điền. Loại buổi: Học / Mini test / Big test. Mốc thông báo: Order in ấn / Order mini test / Order Big Test. Ô UNIT ghi "Unit 1: Tên unit" ở buổi đầu của unit.</t>
+    <t>Mỗi file = 1 chặng của 1 giáo trình. Ô nền vàng là ô cần điền. Loại buổi: Học / Ôn tập / Grammar Basic / Mini test / Big test. Mốc thông báo: Order in ấn / Order mini test / Order Big Test. Ô UNIT ghi "Unit 1: Tên unit" ở buổi đầu của unit; ghi chữ khác (vd. "GRAMMAR BASIC 1 – TOPIC 1", "ÔN TẬP CHẶNG", "BIG TEST") là tiêu đề của riêng buổi đó, buổi vẫn thuộc unit đang học.</t>
   </si>
   <si>
     <t>Chương trình / Giáo trình:</t>
@@ -95,9 +95,15 @@
     <t>Link PPT</t>
   </si>
   <si>
+    <t>Link PPT GVNN</t>
+  </si>
+  <si>
     <t>Link Quizizz</t>
   </si>
   <si>
+    <t>Link Mini test / Kiểm tra từ</t>
+  </si>
+  <si>
     <t>Sản phẩm đầu ra</t>
   </si>
   <si>
@@ -158,6 +164,9 @@
     <t>Order in ấn</t>
   </si>
   <si>
+    <t>Không</t>
+  </si>
+  <si>
     <t>Đồ vật lớp học (bản sửa)</t>
   </si>
   <si>
@@ -191,10 +200,10 @@
     <t>Ảnh gia đình</t>
   </si>
   <si>
-    <t>Mini test</t>
-  </si>
-  <si>
-    <t>Mini test Unit 1–2</t>
+    <t>Ôn tập</t>
+  </si>
+  <si>
+    <t>Ôn tập + Mini test Unit 1–2</t>
   </si>
   <si>
     <t>Đề mini test</t>
@@ -599,7 +608,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:T50"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="true" style="0"/>
@@ -616,23 +625,25 @@
     <col min="12" max="12" width="20" customWidth="true" style="0"/>
     <col min="13" max="13" width="16" customWidth="true" style="0"/>
     <col min="14" max="14" width="16" customWidth="true" style="0"/>
-    <col min="15" max="15" width="24" customWidth="true" style="0"/>
+    <col min="15" max="15" width="16" customWidth="true" style="0"/>
     <col min="16" max="16" width="18" customWidth="true" style="0"/>
-    <col min="17" max="17" width="12" customWidth="true" style="0"/>
-    <col min="18" max="18" width="24" customWidth="true" style="0"/>
+    <col min="17" max="17" width="24" customWidth="true" style="0"/>
+    <col min="18" max="18" width="18" customWidth="true" style="0"/>
+    <col min="19" max="19" width="12" customWidth="true" style="0"/>
+    <col min="20" max="20" width="24" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:20">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:20">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -645,7 +656,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:20">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -659,7 +670,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:20">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -673,7 +684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:20">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -687,7 +698,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:20">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -699,7 +710,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:20">
       <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
@@ -748,8 +759,14 @@
       <c r="R9" s="6" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:18">
+      <c r="S9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -758,19 +775,19 @@
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
@@ -778,214 +795,236 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-    </row>
-    <row r="11" spans="1:18">
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+    </row>
+    <row r="11" spans="1:20">
       <c r="A11" s="7"/>
       <c r="B11" s="7">
         <v>1</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N11" s="8"/>
-      <c r="O11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="P11" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="8"/>
-    </row>
-    <row r="12" spans="1:18">
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="S11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="T11" s="8"/>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12" s="7"/>
       <c r="B12" s="7">
         <v>2</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="N12" s="8"/>
-      <c r="O12" s="8" t="s">
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-    </row>
-    <row r="13" spans="1:18">
+      <c r="T12" s="8"/>
+    </row>
+    <row r="13" spans="1:20">
       <c r="A13" s="7"/>
       <c r="B13" s="7">
         <v>3</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M13" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="N13" s="8"/>
-      <c r="O13" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="P13" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
-    </row>
-    <row r="14" spans="1:18">
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="R13" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="S13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="T13" s="8"/>
+    </row>
+    <row r="14" spans="1:20">
       <c r="A14" s="7"/>
       <c r="B14" s="7">
         <v>4</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N14" s="8"/>
-      <c r="O14" s="8" t="s">
-        <v>57</v>
-      </c>
+      <c r="O14" s="8"/>
       <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
+      <c r="Q14" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="R14" s="8"/>
-    </row>
-    <row r="15" spans="1:18">
+      <c r="S14" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="T14" s="8"/>
+    </row>
+    <row r="15" spans="1:20">
       <c r="A15" s="7"/>
       <c r="B15" s="7">
         <v>5</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
-      <c r="O15" s="8" t="s">
-        <v>60</v>
-      </c>
+      <c r="O15" s="8"/>
       <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
+      <c r="Q15" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="R15" s="8"/>
-    </row>
-    <row r="16" spans="1:18">
+      <c r="S15" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="T15" s="8"/>
+    </row>
+    <row r="16" spans="1:20">
       <c r="A16" s="7"/>
       <c r="B16" s="7">
         <v>6</v>
@@ -1006,8 +1045,10 @@
       <c r="P16" s="8"/>
       <c r="Q16" s="8"/>
       <c r="R16" s="8"/>
-    </row>
-    <row r="17" spans="1:18">
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+    </row>
+    <row r="17" spans="1:20">
       <c r="A17" s="7"/>
       <c r="B17" s="7">
         <v>7</v>
@@ -1028,8 +1069,10 @@
       <c r="P17" s="8"/>
       <c r="Q17" s="8"/>
       <c r="R17" s="8"/>
-    </row>
-    <row r="18" spans="1:18">
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+    </row>
+    <row r="18" spans="1:20">
       <c r="A18" s="7"/>
       <c r="B18" s="7">
         <v>8</v>
@@ -1050,8 +1093,10 @@
       <c r="P18" s="8"/>
       <c r="Q18" s="8"/>
       <c r="R18" s="8"/>
-    </row>
-    <row r="19" spans="1:18">
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+    </row>
+    <row r="19" spans="1:20">
       <c r="A19" s="7"/>
       <c r="B19" s="7">
         <v>9</v>
@@ -1072,8 +1117,10 @@
       <c r="P19" s="8"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
-    </row>
-    <row r="20" spans="1:18">
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+    </row>
+    <row r="20" spans="1:20">
       <c r="A20" s="7"/>
       <c r="B20" s="7">
         <v>10</v>
@@ -1094,8 +1141,10 @@
       <c r="P20" s="8"/>
       <c r="Q20" s="8"/>
       <c r="R20" s="8"/>
-    </row>
-    <row r="21" spans="1:18">
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+    </row>
+    <row r="21" spans="1:20">
       <c r="A21" s="7"/>
       <c r="B21" s="7">
         <v>11</v>
@@ -1116,8 +1165,10 @@
       <c r="P21" s="8"/>
       <c r="Q21" s="8"/>
       <c r="R21" s="8"/>
-    </row>
-    <row r="22" spans="1:18">
+      <c r="S21" s="8"/>
+      <c r="T21" s="8"/>
+    </row>
+    <row r="22" spans="1:20">
       <c r="A22" s="7"/>
       <c r="B22" s="7">
         <v>12</v>
@@ -1138,8 +1189,10 @@
       <c r="P22" s="8"/>
       <c r="Q22" s="8"/>
       <c r="R22" s="8"/>
-    </row>
-    <row r="23" spans="1:18">
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+    </row>
+    <row r="23" spans="1:20">
       <c r="A23" s="7"/>
       <c r="B23" s="7">
         <v>13</v>
@@ -1160,8 +1213,10 @@
       <c r="P23" s="8"/>
       <c r="Q23" s="8"/>
       <c r="R23" s="8"/>
-    </row>
-    <row r="24" spans="1:18">
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+    </row>
+    <row r="24" spans="1:20">
       <c r="A24" s="7"/>
       <c r="B24" s="7">
         <v>14</v>
@@ -1182,8 +1237,10 @@
       <c r="P24" s="8"/>
       <c r="Q24" s="8"/>
       <c r="R24" s="8"/>
-    </row>
-    <row r="25" spans="1:18">
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+    </row>
+    <row r="25" spans="1:20">
       <c r="A25" s="7"/>
       <c r="B25" s="7">
         <v>15</v>
@@ -1204,8 +1261,10 @@
       <c r="P25" s="8"/>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
-    </row>
-    <row r="26" spans="1:18">
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+    </row>
+    <row r="26" spans="1:20">
       <c r="A26" s="7"/>
       <c r="B26" s="7">
         <v>16</v>
@@ -1226,8 +1285,10 @@
       <c r="P26" s="8"/>
       <c r="Q26" s="8"/>
       <c r="R26" s="8"/>
-    </row>
-    <row r="27" spans="1:18">
+      <c r="S26" s="8"/>
+      <c r="T26" s="8"/>
+    </row>
+    <row r="27" spans="1:20">
       <c r="A27" s="7"/>
       <c r="B27" s="7">
         <v>17</v>
@@ -1248,8 +1309,10 @@
       <c r="P27" s="8"/>
       <c r="Q27" s="8"/>
       <c r="R27" s="8"/>
-    </row>
-    <row r="28" spans="1:18">
+      <c r="S27" s="8"/>
+      <c r="T27" s="8"/>
+    </row>
+    <row r="28" spans="1:20">
       <c r="A28" s="7"/>
       <c r="B28" s="7">
         <v>18</v>
@@ -1270,8 +1333,10 @@
       <c r="P28" s="8"/>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
-    </row>
-    <row r="29" spans="1:18">
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
+    </row>
+    <row r="29" spans="1:20">
       <c r="A29" s="7"/>
       <c r="B29" s="7">
         <v>19</v>
@@ -1292,8 +1357,10 @@
       <c r="P29" s="8"/>
       <c r="Q29" s="8"/>
       <c r="R29" s="8"/>
-    </row>
-    <row r="30" spans="1:18">
+      <c r="S29" s="8"/>
+      <c r="T29" s="8"/>
+    </row>
+    <row r="30" spans="1:20">
       <c r="A30" s="7"/>
       <c r="B30" s="7">
         <v>20</v>
@@ -1314,8 +1381,10 @@
       <c r="P30" s="8"/>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
-    </row>
-    <row r="31" spans="1:18">
+      <c r="S30" s="8"/>
+      <c r="T30" s="8"/>
+    </row>
+    <row r="31" spans="1:20">
       <c r="A31" s="7"/>
       <c r="B31" s="7">
         <v>21</v>
@@ -1336,8 +1405,10 @@
       <c r="P31" s="8"/>
       <c r="Q31" s="8"/>
       <c r="R31" s="8"/>
-    </row>
-    <row r="32" spans="1:18">
+      <c r="S31" s="8"/>
+      <c r="T31" s="8"/>
+    </row>
+    <row r="32" spans="1:20">
       <c r="A32" s="7"/>
       <c r="B32" s="7">
         <v>22</v>
@@ -1358,8 +1429,10 @@
       <c r="P32" s="8"/>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
-    </row>
-    <row r="33" spans="1:18">
+      <c r="S32" s="8"/>
+      <c r="T32" s="8"/>
+    </row>
+    <row r="33" spans="1:20">
       <c r="A33" s="7"/>
       <c r="B33" s="7">
         <v>23</v>
@@ -1380,8 +1453,10 @@
       <c r="P33" s="8"/>
       <c r="Q33" s="8"/>
       <c r="R33" s="8"/>
-    </row>
-    <row r="34" spans="1:18">
+      <c r="S33" s="8"/>
+      <c r="T33" s="8"/>
+    </row>
+    <row r="34" spans="1:20">
       <c r="A34" s="7"/>
       <c r="B34" s="7">
         <v>24</v>
@@ -1402,8 +1477,10 @@
       <c r="P34" s="8"/>
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
-    </row>
-    <row r="35" spans="1:18">
+      <c r="S34" s="8"/>
+      <c r="T34" s="8"/>
+    </row>
+    <row r="35" spans="1:20">
       <c r="A35" s="7"/>
       <c r="B35" s="7">
         <v>25</v>
@@ -1424,8 +1501,10 @@
       <c r="P35" s="8"/>
       <c r="Q35" s="8"/>
       <c r="R35" s="8"/>
-    </row>
-    <row r="36" spans="1:18">
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+    </row>
+    <row r="36" spans="1:20">
       <c r="A36" s="7"/>
       <c r="B36" s="7">
         <v>26</v>
@@ -1446,8 +1525,10 @@
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
       <c r="R36" s="8"/>
-    </row>
-    <row r="37" spans="1:18">
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+    </row>
+    <row r="37" spans="1:20">
       <c r="A37" s="7"/>
       <c r="B37" s="7">
         <v>27</v>
@@ -1468,8 +1549,10 @@
       <c r="P37" s="8"/>
       <c r="Q37" s="8"/>
       <c r="R37" s="8"/>
-    </row>
-    <row r="38" spans="1:18">
+      <c r="S37" s="8"/>
+      <c r="T37" s="8"/>
+    </row>
+    <row r="38" spans="1:20">
       <c r="A38" s="7"/>
       <c r="B38" s="7">
         <v>28</v>
@@ -1490,8 +1573,10 @@
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8"/>
-    </row>
-    <row r="39" spans="1:18">
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+    </row>
+    <row r="39" spans="1:20">
       <c r="A39" s="7"/>
       <c r="B39" s="7">
         <v>29</v>
@@ -1512,8 +1597,10 @@
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
       <c r="R39" s="8"/>
-    </row>
-    <row r="40" spans="1:18">
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+    </row>
+    <row r="40" spans="1:20">
       <c r="A40" s="7"/>
       <c r="B40" s="7">
         <v>30</v>
@@ -1534,8 +1621,10 @@
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
       <c r="R40" s="8"/>
-    </row>
-    <row r="41" spans="1:18">
+      <c r="S40" s="8"/>
+      <c r="T40" s="8"/>
+    </row>
+    <row r="41" spans="1:20">
       <c r="A41" s="7"/>
       <c r="B41" s="7">
         <v>31</v>
@@ -1556,8 +1645,10 @@
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
       <c r="R41" s="8"/>
-    </row>
-    <row r="42" spans="1:18">
+      <c r="S41" s="8"/>
+      <c r="T41" s="8"/>
+    </row>
+    <row r="42" spans="1:20">
       <c r="A42" s="7"/>
       <c r="B42" s="7">
         <v>32</v>
@@ -1578,8 +1669,10 @@
       <c r="P42" s="8"/>
       <c r="Q42" s="8"/>
       <c r="R42" s="8"/>
-    </row>
-    <row r="43" spans="1:18">
+      <c r="S42" s="8"/>
+      <c r="T42" s="8"/>
+    </row>
+    <row r="43" spans="1:20">
       <c r="A43" s="7"/>
       <c r="B43" s="7">
         <v>33</v>
@@ -1600,8 +1693,10 @@
       <c r="P43" s="8"/>
       <c r="Q43" s="8"/>
       <c r="R43" s="8"/>
-    </row>
-    <row r="44" spans="1:18">
+      <c r="S43" s="8"/>
+      <c r="T43" s="8"/>
+    </row>
+    <row r="44" spans="1:20">
       <c r="A44" s="7"/>
       <c r="B44" s="7">
         <v>34</v>
@@ -1622,8 +1717,10 @@
       <c r="P44" s="8"/>
       <c r="Q44" s="8"/>
       <c r="R44" s="8"/>
-    </row>
-    <row r="45" spans="1:18">
+      <c r="S44" s="8"/>
+      <c r="T44" s="8"/>
+    </row>
+    <row r="45" spans="1:20">
       <c r="A45" s="7"/>
       <c r="B45" s="7">
         <v>35</v>
@@ -1644,8 +1741,10 @@
       <c r="P45" s="8"/>
       <c r="Q45" s="8"/>
       <c r="R45" s="8"/>
-    </row>
-    <row r="46" spans="1:18">
+      <c r="S45" s="8"/>
+      <c r="T45" s="8"/>
+    </row>
+    <row r="46" spans="1:20">
       <c r="A46" s="7"/>
       <c r="B46" s="7">
         <v>36</v>
@@ -1666,8 +1765,10 @@
       <c r="P46" s="8"/>
       <c r="Q46" s="8"/>
       <c r="R46" s="8"/>
-    </row>
-    <row r="47" spans="1:18">
+      <c r="S46" s="8"/>
+      <c r="T46" s="8"/>
+    </row>
+    <row r="47" spans="1:20">
       <c r="A47" s="7"/>
       <c r="B47" s="7">
         <v>37</v>
@@ -1688,8 +1789,10 @@
       <c r="P47" s="8"/>
       <c r="Q47" s="8"/>
       <c r="R47" s="8"/>
-    </row>
-    <row r="48" spans="1:18">
+      <c r="S47" s="8"/>
+      <c r="T47" s="8"/>
+    </row>
+    <row r="48" spans="1:20">
       <c r="A48" s="7"/>
       <c r="B48" s="7">
         <v>38</v>
@@ -1710,8 +1813,10 @@
       <c r="P48" s="8"/>
       <c r="Q48" s="8"/>
       <c r="R48" s="8"/>
-    </row>
-    <row r="49" spans="1:18">
+      <c r="S48" s="8"/>
+      <c r="T48" s="8"/>
+    </row>
+    <row r="49" spans="1:20">
       <c r="A49" s="7"/>
       <c r="B49" s="7">
         <v>39</v>
@@ -1732,8 +1837,10 @@
       <c r="P49" s="8"/>
       <c r="Q49" s="8"/>
       <c r="R49" s="8"/>
-    </row>
-    <row r="50" spans="1:18">
+      <c r="S49" s="8"/>
+      <c r="T49" s="8"/>
+    </row>
+    <row r="50" spans="1:20">
       <c r="A50" s="7"/>
       <c r="B50" s="7">
         <v>40</v>
@@ -1754,6 +1861,8 @@
       <c r="P50" s="8"/>
       <c r="Q50" s="8"/>
       <c r="R50" s="8"/>
+      <c r="S50" s="8"/>
+      <c r="T50" s="8"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>